<commit_message>
MinComplinace with mass and cost constraint: LBracket with 3 materials (temperature dependent) working
</commit_message>
<xml_diff>
--- a/DataConstantTemperature/BridgeMaterials.xlsx
+++ b/DataConstantTemperature/BridgeMaterials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ksure\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataConstantTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C038D72-A43F-46D0-BAD5-4D5A22BC6BF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC93697F-FAAD-4797-A225-0102CE188221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2964" yWindow="2964" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-3030" yWindow="2270" windowWidth="19200" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -525,14 +525,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" style="10" customWidth="1"/>
-    <col min="2" max="702" width="20.5546875" style="10" customWidth="1"/>
-    <col min="703" max="16384" width="9.109375" style="10"/>
+    <col min="1" max="1" width="20.6328125" style="10" customWidth="1"/>
+    <col min="2" max="702" width="20.54296875" style="10" customWidth="1"/>
+    <col min="703" max="16384" width="9.08984375" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>17</v>
       </c>
@@ -546,7 +546,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
         <v>18</v>
       </c>
@@ -560,7 +560,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>19</v>
       </c>
@@ -574,7 +574,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>20</v>
       </c>
@@ -588,7 +588,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>21</v>
       </c>
@@ -627,12 +627,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC80EBF-8B96-4896-8C13-AD8A976D05A3}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -646,7 +646,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -660,7 +660,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -674,7 +674,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -688,7 +688,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>

</xml_diff>